<commit_message>
Maj streamlit topic modeling
</commit_message>
<xml_diff>
--- a/data/labelled_topics/topics_top_words_phrases_annoté.xlsx
+++ b/data/labelled_topics/topics_top_words_phrases_annoté.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charb\Documents\ALTERNANCE\Datascientest\Projet\TrustPilot\DS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charb\Documents\ALTERNANCE\Datascientest\Projet\TrustPilot\DS\nov24_alt_trustpilot\data\labelled_topics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551668EB-FEA9-4B55-BEC8-E560640963D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3403B52-8498-4F83-ABD6-C142A7EFB178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{A5B3868A-FEAE-403F-8DCD-09EB72FD6FE8}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="447">
   <si>
     <t>Topic</t>
   </si>
@@ -1387,9 +1387,6 @@
   </si>
   <si>
     <t>Qualité produit / Livraison</t>
-  </si>
-  <si>
-    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -1507,11 +1504,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E06E303F-7458-4B98-A4EE-0FE27C79FC6E}" name="topics_top_words_phrases" displayName="topics_top_words_phrases" ref="A1:F203" tableType="queryTable" totalsRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E06E303F-7458-4B98-A4EE-0FE27C79FC6E}" name="topics_top_words_phrases" displayName="topics_top_words_phrases" ref="A1:F202" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:F202" xr:uid="{E06E303F-7458-4B98-A4EE-0FE27C79FC6E}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{FFE0BAFE-C04A-4A31-AC4A-912309F76E36}" uniqueName="1" name="Topic" totalsRowLabel="Total" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{7D5094E6-1A33-487D-8D28-DEDC1F66C6F9}" uniqueName="2" name="Count" totalsRowFunction="sum" queryTableFieldId="2"/>
+    <tableColumn id="1" xr3:uid="{FFE0BAFE-C04A-4A31-AC4A-912309F76E36}" uniqueName="1" name="Topic" queryTableFieldId="1"/>
+    <tableColumn id="2" xr3:uid="{7D5094E6-1A33-487D-8D28-DEDC1F66C6F9}" uniqueName="2" name="Count" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{9A7564D2-263D-45ED-8DD7-08A0E3C8B586}" uniqueName="3" name="Name" queryTableFieldId="3" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{F53DF144-B85D-4E5E-A0BD-76B8C121B92D}" uniqueName="4" name="Representation" queryTableFieldId="4" dataDxfId="2"/>
     <tableColumn id="5" xr3:uid="{6642FB0F-A6E2-4E40-9FEC-B2890B820381}" uniqueName="5" name="Representative_Docs" queryTableFieldId="5" dataDxfId="1"/>
@@ -1838,7 +1835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{548FE5B4-2897-4FA5-9050-631E1572915F}">
-  <dimension ref="A1:F203"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="7.73046875" bestFit="1" customWidth="1"/>
@@ -5884,15 +5881,6 @@
       </c>
       <c r="F202" t="s">
         <v>446</v>
-      </c>
-    </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A203" t="s">
-        <v>447</v>
-      </c>
-      <c r="B203">
-        <f>SUBTOTAL(109,topics_top_words_phrases[Count])</f>
-        <v>37628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>